<commit_message>
updated ARR in RTM
</commit_message>
<xml_diff>
--- a/Requirements-Analysis/Requirments-Traceability-Matrix.xlsx
+++ b/Requirements-Analysis/Requirments-Traceability-Matrix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chitrangidoshi/Documents/Buisness Analyst/Case Study/Tiimo/Requirement Analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chitrangidoshi/Documents/Buisness Analyst/Case Study/Tiimo/github repo/Tiimo-Case-Study/Requirements-Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADB94DA5-E701-BC4D-BBA7-D18186F68695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621E462D-E0FE-2145-846E-51F5F0BDE1A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{3BB15FB3-0FC9-1E40-AC92-8B092F7CE3D8}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15740" xr2:uid="{3BB15FB3-0FC9-1E40-AC92-8B092F7CE3D8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -221,9 +221,6 @@
     <t>BR-01, SR-04</t>
   </si>
   <si>
-    <t>Analysis of 113 low-rating iPhone reviews shows Routines complaints in 25 cases (22% of total), with 19.2% explicit churn signals like cancellations. Example: "Wish they would bring back routines...helps me flow" (ASNZ001 Affinity_Traceability_Analysis_Tiimo.xlsx​). Calendar sync bugs in 9 reviews also contribute to churn VOC-Analysis.xlsx​.</t>
-  </si>
-  <si>
     <t>VOC Evidence</t>
   </si>
   <si>
@@ -438,6 +435,9 @@
   </si>
   <si>
     <t>REQUIREMENTS TRACEABILITY MATRIX - TIIMO IPHONE CHURN REDUCTION</t>
+  </si>
+  <si>
+    <t>Analysis of 113 low-rating iPhone reviews shows Routines complaints in 25 cases (22% of total), with 13.5% explicit churn signals like cancellations costing Tiimo approx $119K. Example: "Wish they would bring back routines...helps me flow" (ASNZ001 Affinity_Traceability_Analysis_Tiimo.xlsx​). Calendar sync bugs in 9 reviews also contribute to churn VOC-Analysis.xlsx​.</t>
   </si>
 </sst>
 </file>
@@ -445,7 +445,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -642,10 +642,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -704,7 +704,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="168" formatCode="0.0"/>
+      <numFmt numFmtId="164" formatCode="0.0"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
@@ -968,13 +968,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color indexed="64"/>
@@ -1008,6 +1001,13 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1063,7 +1063,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{963E5FD2-6E35-AD43-966F-AB3183845483}" name="Table_RTM" displayName="Table_RTM" ref="A5:I28" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12" headerRowBorderDxfId="10" tableBorderDxfId="11" totalsRowBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{963E5FD2-6E35-AD43-966F-AB3183845483}" name="Table_RTM" displayName="Table_RTM" ref="A5:I28" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10" totalsRowBorderDxfId="9">
   <autoFilter ref="A5:I28" xr:uid="{963E5FD2-6E35-AD43-966F-AB3183845483}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:I28">
     <sortCondition ref="A5:A28"/>
@@ -1415,7 +1415,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1470,7 +1470,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>3</v>
@@ -1497,16 +1497,16 @@
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
-        <v>61</v>
+        <v>133</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H6" s="9">
         <v>30</v>
@@ -1524,16 +1524,16 @@
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H7" s="10">
         <v>20</v>
@@ -1553,16 +1553,16 @@
         <v>58</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H8" s="9">
         <v>60</v>
@@ -1582,16 +1582,16 @@
         <v>58</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H9" s="9">
         <v>60</v>
@@ -1611,16 +1611,16 @@
         <v>59</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H10" s="9">
         <v>48.6</v>
@@ -1640,16 +1640,16 @@
         <v>60</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H11" s="9">
         <v>32.4</v>
@@ -1669,16 +1669,16 @@
         <v>58</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H12" s="9">
         <v>28.8</v>
@@ -1698,16 +1698,16 @@
         <v>40</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H13" s="9">
         <v>30.375</v>
@@ -1727,16 +1727,16 @@
         <v>34</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H14" s="9">
         <v>29.4</v>
@@ -1756,16 +1756,16 @@
         <v>10</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H15" s="9">
         <v>54</v>
@@ -1785,16 +1785,16 @@
         <v>10</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H16" s="9">
         <v>48</v>
@@ -1814,16 +1814,16 @@
         <v>8</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H17" s="9">
         <v>60</v>
@@ -1843,16 +1843,16 @@
         <v>38</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>110</v>
-      </c>
       <c r="G18" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H18" s="9">
         <v>57.6</v>
@@ -1872,16 +1872,16 @@
         <v>8</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H19" s="9">
         <v>36</v>
@@ -1901,16 +1901,16 @@
         <v>57</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H20" s="9">
         <v>14.4</v>
@@ -1930,16 +1930,16 @@
         <v>8</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="F21" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H21" s="9">
         <v>32.4</v>
@@ -1959,16 +1959,16 @@
         <v>55</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H22" s="9">
         <v>38.4</v>
@@ -1988,16 +1988,16 @@
         <v>34</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H23" s="9">
         <v>34.299999999999997</v>
@@ -2017,16 +2017,16 @@
         <v>53</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H24" s="9">
         <v>57.6</v>
@@ -2046,16 +2046,16 @@
         <v>8</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H25" s="9">
         <v>22.399999999999995</v>
@@ -2075,16 +2075,16 @@
         <v>8</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H26" s="9">
         <v>22.049999999999997</v>
@@ -2104,16 +2104,16 @@
         <v>53</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H27" s="9">
         <v>42</v>
@@ -2133,16 +2133,16 @@
         <v>53</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H28" s="9">
         <v>51.2</v>

</xml_diff>